<commit_message>
chore: publish upm packages (7 packages)
Published packages:
- com.solotopia.nova.framework@0.5.35
- com.solotopia.nova.framework.sdk.appsflyer@0.0.22
- com.solotopia.nova.framework.sdk.datamaster.abtest@0.0.2
- com.solotopia.nova.framework.sdk.facebook@0.0.5
- com.solotopia.nova.framework.sdk.firebase@0.0.20
- com.solotopia.nova.framework.sdk.googlesignin@0.0.3
- com.solotopia.nova.framework.sdk.tga@0.0.18
</commit_message>
<xml_diff>
--- a/Assets/Samples/AppleSigninDemo/Excels/Networks/HostKeys/NetworkHostKeys.xlsx
+++ b/Assets/Samples/AppleSigninDemo/Excels/Networks/HostKeys/NetworkHostKeys.xlsx
@@ -1,256 +1,191 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="26860" windowHeight="12660"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="26860" windowHeight="12660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="NetworkHostKeys" sheetId="1" r:id="rId1"/>
+    <sheet name="NetworkHostKeys" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="14">
-  <si>
-    <t>##comment</t>
-  </si>
-  <si>
-    <t>网络域名表（NetHosts）</t>
-  </si>
-  <si>
-    <t>##var</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>#Desc</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>##type</t>
-  </si>
-  <si>
-    <t>string</t>
-  </si>
-  <si>
-    <t>主机唯一标识名</t>
-  </si>
-  <si>
-    <t>描述</t>
-  </si>
-  <si>
-    <t>URL</t>
-  </si>
-  <si>
-    <t>TGAServer</t>
-  </si>
-  <si>
-    <t>游戏服务器url前缀</t>
-  </si>
-  <si>
-    <t>https://report.lolipopmobi.com</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="22">
     <font>
-      <sz val="11"/>
+      <name val="宋体"/>
+      <charset val="134"/>
       <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
+      <color rgb="FF000000"/>
       <sz val="9.75"/>
-      <color rgb="FF000000"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
+      <color rgb="FFFFFFFF"/>
       <sz val="9.75"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF800080"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="18"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <i val="1"/>
+      <color rgb="FF7F7F7F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="15"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="13"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF3F3F76"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FF3F3F3F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
       <color rgb="FFFFFFFF"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
+      <color rgb="FF006100"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <color rgb="FF9C0006"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FF9C6500"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color theme="0"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="38">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -609,169 +544,169 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="35" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="36" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="37" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="7">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -827,11 +762,74 @@
     <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -1118,143 +1116,196 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:X41"/>
-  <sheetFormatPr defaultColWidth="13" defaultRowHeight="16.8"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:X6"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="13" defaultRowHeight="16.8"/>
   <cols>
-    <col min="1" max="1" width="12" style="1" customWidth="1"/>
-    <col min="2" max="2" width="37" style="2" customWidth="1"/>
-    <col min="3" max="3" width="44.8461538461538" style="2" customWidth="1"/>
-    <col min="4" max="4" width="95" style="2" customWidth="1"/>
-    <col min="5" max="24" width="37" style="2" customWidth="1"/>
-    <col min="25" max="16384" width="13" style="3"/>
+    <col width="12" customWidth="1" style="1" min="1" max="1"/>
+    <col width="37" customWidth="1" style="2" min="2" max="2"/>
+    <col width="44.8461538461538" customWidth="1" style="2" min="3" max="3"/>
+    <col width="95" customWidth="1" style="2" min="4" max="4"/>
+    <col width="37" customWidth="1" style="2" min="5" max="24"/>
+    <col width="13" customWidth="1" style="3" min="25" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:24">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
-      <c r="P1" s="4"/>
-      <c r="Q1" s="4"/>
-      <c r="R1" s="4"/>
-      <c r="S1" s="4"/>
-      <c r="T1" s="4"/>
-      <c r="U1" s="4"/>
-      <c r="V1" s="4"/>
-      <c r="W1" s="4"/>
-      <c r="X1" s="4"/>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>##comment</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>网络域名表（NetHosts）</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="n"/>
+      <c r="D1" s="4" t="n"/>
+      <c r="E1" s="4" t="n"/>
+      <c r="F1" s="4" t="n"/>
+      <c r="G1" s="4" t="n"/>
+      <c r="H1" s="4" t="n"/>
+      <c r="I1" s="4" t="n"/>
+      <c r="J1" s="4" t="n"/>
+      <c r="K1" s="4" t="n"/>
+      <c r="L1" s="4" t="n"/>
+      <c r="M1" s="4" t="n"/>
+      <c r="N1" s="4" t="n"/>
+      <c r="O1" s="4" t="n"/>
+      <c r="P1" s="4" t="n"/>
+      <c r="Q1" s="4" t="n"/>
+      <c r="R1" s="4" t="n"/>
+      <c r="S1" s="4" t="n"/>
+      <c r="T1" s="4" t="n"/>
+      <c r="U1" s="4" t="n"/>
+      <c r="V1" s="4" t="n"/>
+      <c r="W1" s="4" t="n"/>
+      <c r="X1" s="4" t="n"/>
     </row>
-    <row r="2" ht="22" customHeight="1" spans="1:24">
-      <c r="A2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
-      <c r="J2" s="5"/>
-      <c r="K2" s="5"/>
-      <c r="L2" s="5"/>
-      <c r="M2" s="5"/>
-      <c r="N2" s="5"/>
-      <c r="O2" s="5"/>
-      <c r="P2" s="5"/>
-      <c r="Q2" s="5"/>
-      <c r="R2" s="5"/>
-      <c r="S2" s="5"/>
-      <c r="T2" s="5"/>
-      <c r="U2" s="5"/>
-      <c r="V2" s="5"/>
-      <c r="W2" s="5"/>
-      <c r="X2" s="5"/>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>##var</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>#Desc</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="n"/>
+      <c r="F2" s="5" t="n"/>
+      <c r="G2" s="5" t="n"/>
+      <c r="H2" s="5" t="n"/>
+      <c r="I2" s="5" t="n"/>
+      <c r="J2" s="5" t="n"/>
+      <c r="K2" s="5" t="n"/>
+      <c r="L2" s="5" t="n"/>
+      <c r="M2" s="5" t="n"/>
+      <c r="N2" s="5" t="n"/>
+      <c r="O2" s="5" t="n"/>
+      <c r="P2" s="5" t="n"/>
+      <c r="Q2" s="5" t="n"/>
+      <c r="R2" s="5" t="n"/>
+      <c r="S2" s="5" t="n"/>
+      <c r="T2" s="5" t="n"/>
+      <c r="U2" s="5" t="n"/>
+      <c r="V2" s="5" t="n"/>
+      <c r="W2" s="5" t="n"/>
+      <c r="X2" s="5" t="n"/>
     </row>
-    <row r="3" ht="22" customHeight="1" spans="1:24">
-      <c r="A3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
-      <c r="K3" s="6"/>
-      <c r="L3" s="6"/>
-      <c r="M3" s="6"/>
-      <c r="N3" s="6"/>
-      <c r="O3" s="6"/>
-      <c r="P3" s="6"/>
-      <c r="Q3" s="6"/>
-      <c r="R3" s="6"/>
-      <c r="S3" s="6"/>
-      <c r="T3" s="6"/>
-      <c r="U3" s="6"/>
-      <c r="V3" s="6"/>
-      <c r="W3" s="6"/>
-      <c r="X3" s="6"/>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>##type</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="6" t="n"/>
+      <c r="G3" s="6" t="n"/>
+      <c r="H3" s="6" t="n"/>
+      <c r="I3" s="6" t="n"/>
+      <c r="J3" s="6" t="n"/>
+      <c r="K3" s="6" t="n"/>
+      <c r="L3" s="6" t="n"/>
+      <c r="M3" s="6" t="n"/>
+      <c r="N3" s="6" t="n"/>
+      <c r="O3" s="6" t="n"/>
+      <c r="P3" s="6" t="n"/>
+      <c r="Q3" s="6" t="n"/>
+      <c r="R3" s="6" t="n"/>
+      <c r="S3" s="6" t="n"/>
+      <c r="T3" s="6" t="n"/>
+      <c r="U3" s="6" t="n"/>
+      <c r="V3" s="6" t="n"/>
+      <c r="W3" s="6" t="n"/>
+      <c r="X3" s="6" t="n"/>
     </row>
-    <row r="4" s="1" customFormat="1" ht="22" customHeight="1" spans="1:24">
-      <c r="A4" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>10</v>
+    <row r="4" ht="22" customFormat="1" customHeight="1" s="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>##comment</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>主机唯一标识名</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>描述</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
       </c>
     </row>
-    <row r="5" ht="22" customHeight="1" spans="1:24">
-      <c r="B5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>13</v>
+    <row r="5" ht="22" customHeight="1">
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>TGAServer</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>游戏服务器url前缀</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>https://report.lolipopmobi.com</t>
+        </is>
       </c>
     </row>
-    <row r="6" ht="22" customHeight="1"/>
+    <row r="6" ht="22" customHeight="1">
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>GameServer</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>游戏服务器url前缀</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>https://t-solo-api-game.ahameet.com</t>
+        </is>
+      </c>
+    </row>
     <row r="7" ht="22" customHeight="1"/>
     <row r="8" ht="22" customHeight="1"/>
     <row r="9" ht="22" customHeight="1"/>
@@ -1292,6 +1343,5 @@
     <row r="41" ht="22" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: sync Nova upm-release-2026.07.23-02
</commit_message>
<xml_diff>
--- a/Assets/Samples/AppleSigninDemo/Excels/Networks/HostKeys/NetworkHostKeys.xlsx
+++ b/Assets/Samples/AppleSigninDemo/Excels/Networks/HostKeys/NetworkHostKeys.xlsx
@@ -6,7 +6,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="26860" windowHeight="12660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="NetworkHostKeys" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="NetworkHostKeys-Debug" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="NetworkHostKeys-Release" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1344,4 +1345,235 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:X6"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="13" defaultRowHeight="16.8"/>
+  <cols>
+    <col width="12" customWidth="1" style="1" min="1" max="1"/>
+    <col width="37" customWidth="1" style="2" min="2" max="2"/>
+    <col width="44.8461538461538" customWidth="1" style="2" min="3" max="3"/>
+    <col width="95" customWidth="1" style="2" min="4" max="4"/>
+    <col width="37" customWidth="1" style="2" min="5" max="24"/>
+    <col width="13" customWidth="1" style="3" min="25" max="16384"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>##comment</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>网络域名表（NetHosts）</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="n"/>
+      <c r="D1" s="4" t="n"/>
+      <c r="E1" s="4" t="n"/>
+      <c r="F1" s="4" t="n"/>
+      <c r="G1" s="4" t="n"/>
+      <c r="H1" s="4" t="n"/>
+      <c r="I1" s="4" t="n"/>
+      <c r="J1" s="4" t="n"/>
+      <c r="K1" s="4" t="n"/>
+      <c r="L1" s="4" t="n"/>
+      <c r="M1" s="4" t="n"/>
+      <c r="N1" s="4" t="n"/>
+      <c r="O1" s="4" t="n"/>
+      <c r="P1" s="4" t="n"/>
+      <c r="Q1" s="4" t="n"/>
+      <c r="R1" s="4" t="n"/>
+      <c r="S1" s="4" t="n"/>
+      <c r="T1" s="4" t="n"/>
+      <c r="U1" s="4" t="n"/>
+      <c r="V1" s="4" t="n"/>
+      <c r="W1" s="4" t="n"/>
+      <c r="X1" s="4" t="n"/>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>##var</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>#Desc</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="n"/>
+      <c r="F2" s="5" t="n"/>
+      <c r="G2" s="5" t="n"/>
+      <c r="H2" s="5" t="n"/>
+      <c r="I2" s="5" t="n"/>
+      <c r="J2" s="5" t="n"/>
+      <c r="K2" s="5" t="n"/>
+      <c r="L2" s="5" t="n"/>
+      <c r="M2" s="5" t="n"/>
+      <c r="N2" s="5" t="n"/>
+      <c r="O2" s="5" t="n"/>
+      <c r="P2" s="5" t="n"/>
+      <c r="Q2" s="5" t="n"/>
+      <c r="R2" s="5" t="n"/>
+      <c r="S2" s="5" t="n"/>
+      <c r="T2" s="5" t="n"/>
+      <c r="U2" s="5" t="n"/>
+      <c r="V2" s="5" t="n"/>
+      <c r="W2" s="5" t="n"/>
+      <c r="X2" s="5" t="n"/>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>##type</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="6" t="n"/>
+      <c r="G3" s="6" t="n"/>
+      <c r="H3" s="6" t="n"/>
+      <c r="I3" s="6" t="n"/>
+      <c r="J3" s="6" t="n"/>
+      <c r="K3" s="6" t="n"/>
+      <c r="L3" s="6" t="n"/>
+      <c r="M3" s="6" t="n"/>
+      <c r="N3" s="6" t="n"/>
+      <c r="O3" s="6" t="n"/>
+      <c r="P3" s="6" t="n"/>
+      <c r="Q3" s="6" t="n"/>
+      <c r="R3" s="6" t="n"/>
+      <c r="S3" s="6" t="n"/>
+      <c r="T3" s="6" t="n"/>
+      <c r="U3" s="6" t="n"/>
+      <c r="V3" s="6" t="n"/>
+      <c r="W3" s="6" t="n"/>
+      <c r="X3" s="6" t="n"/>
+    </row>
+    <row r="4" ht="22" customFormat="1" customHeight="1" s="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>##comment</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>主机唯一标识名</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>描述</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>TGAServer</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>游戏服务器url前缀</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>https://report.lolipopmobi.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>GameServer</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>游戏服务器url前缀</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>https://t-solo-api-game.ahameet.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1"/>
+    <row r="8" ht="22" customHeight="1"/>
+    <row r="9" ht="22" customHeight="1"/>
+    <row r="10" ht="22" customHeight="1"/>
+    <row r="11" ht="22" customHeight="1"/>
+    <row r="12" ht="22" customHeight="1"/>
+    <row r="13" ht="22" customHeight="1"/>
+    <row r="14" ht="22" customHeight="1"/>
+    <row r="15" ht="22" customHeight="1"/>
+    <row r="16" ht="22" customHeight="1"/>
+    <row r="17" ht="22" customHeight="1"/>
+    <row r="18" ht="22" customHeight="1"/>
+    <row r="19" ht="22" customHeight="1"/>
+    <row r="20" ht="22" customHeight="1"/>
+    <row r="21" ht="22" customHeight="1"/>
+    <row r="22" ht="22" customHeight="1"/>
+    <row r="23" ht="22" customHeight="1"/>
+    <row r="24" ht="22" customHeight="1"/>
+    <row r="25" ht="22" customHeight="1"/>
+    <row r="26" ht="22" customHeight="1"/>
+    <row r="27" ht="22" customHeight="1"/>
+    <row r="28" ht="22" customHeight="1"/>
+    <row r="29" ht="22" customHeight="1"/>
+    <row r="30" ht="22" customHeight="1"/>
+    <row r="31" ht="22" customHeight="1"/>
+    <row r="32" ht="22" customHeight="1"/>
+    <row r="33" ht="22" customHeight="1"/>
+    <row r="34" ht="22" customHeight="1"/>
+    <row r="35" ht="22" customHeight="1"/>
+    <row r="36" ht="22" customHeight="1"/>
+    <row r="37" ht="22" customHeight="1"/>
+    <row r="38" ht="22" customHeight="1"/>
+    <row r="39" ht="22" customHeight="1"/>
+    <row r="40" ht="22" customHeight="1"/>
+    <row r="41" ht="22" customHeight="1"/>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>